<commit_message>
fix bugs with trial ending earlier
</commit_message>
<xml_diff>
--- a/Trials.xlsx
+++ b/Trials.xlsx
@@ -1,32 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20395"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20397"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PMDLAB\Documents\Python-Experiments\Visuomotor-Rotation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PMDLAB\Documents\Python-Experiments\psychopy-scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{895BD332-0346-49E3-919F-050083D52CAC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F631AF2D-7927-4D20-8512-F542B306A450}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="5" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="7" r:id="rId2"/>
-    <sheet name="Testing" sheetId="6" r:id="rId3"/>
-    <sheet name="Practice" sheetId="1" r:id="rId4"/>
-    <sheet name="Baseline" sheetId="2" r:id="rId5"/>
-    <sheet name="Exposure" sheetId="3" r:id="rId6"/>
-    <sheet name="Post" sheetId="4" r:id="rId7"/>
+    <sheet name="Testing" sheetId="6" r:id="rId2"/>
+    <sheet name="Practice" sheetId="1" r:id="rId3"/>
+    <sheet name="Baseline" sheetId="2" r:id="rId4"/>
+    <sheet name="Exposure" sheetId="3" r:id="rId5"/>
+    <sheet name="Post" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="25">
   <si>
     <t>trial_num</t>
   </si>
@@ -111,9 +110,6 @@
   <si>
     <t>Vibration = 1
 No Vibration = 0</t>
-  </si>
-  <si>
-    <t>Targets</t>
   </si>
 </sst>
 </file>
@@ -701,46 +697,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C2E2371-4466-45A3-B19E-D14944398B7C}">
-  <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="15.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>135</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE99B65C-ABAC-4777-BF85-4382D600E37D}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5703125" style="3" bestFit="1" customWidth="1"/>
@@ -881,10 +842,10 @@
         <v>0</v>
       </c>
       <c r="G4" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="14">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I4" s="14">
         <v>0</v>
@@ -916,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="G5" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" s="14">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I5" s="14">
         <v>0</v>
@@ -929,146 +890,6 @@
       </c>
       <c r="K5" s="14">
         <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>45</v>
-      </c>
-      <c r="C6" s="1">
-        <v>3</v>
-      </c>
-      <c r="D6" s="1">
-        <v>1</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6" s="14">
-        <v>0</v>
-      </c>
-      <c r="G6" s="14">
-        <v>0</v>
-      </c>
-      <c r="H6" s="14">
-        <v>0</v>
-      </c>
-      <c r="I6" s="14">
-        <v>0</v>
-      </c>
-      <c r="J6" s="14">
-        <v>0</v>
-      </c>
-      <c r="K6" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>75</v>
-      </c>
-      <c r="C7" s="1">
-        <v>3</v>
-      </c>
-      <c r="D7" s="1">
-        <v>1</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7" s="14">
-        <v>0</v>
-      </c>
-      <c r="G7" s="14">
-        <v>0</v>
-      </c>
-      <c r="H7" s="14">
-        <v>0</v>
-      </c>
-      <c r="I7" s="14">
-        <v>0</v>
-      </c>
-      <c r="J7" s="14">
-        <v>0</v>
-      </c>
-      <c r="K7" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>105</v>
-      </c>
-      <c r="C8" s="1">
-        <v>3</v>
-      </c>
-      <c r="D8" s="1">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8" s="14">
-        <v>0</v>
-      </c>
-      <c r="G8" s="14">
-        <v>0</v>
-      </c>
-      <c r="H8" s="14">
-        <v>0</v>
-      </c>
-      <c r="I8" s="14">
-        <v>0</v>
-      </c>
-      <c r="J8" s="14">
-        <v>0</v>
-      </c>
-      <c r="K8" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>135</v>
-      </c>
-      <c r="C9" s="1">
-        <v>3</v>
-      </c>
-      <c r="D9" s="1">
-        <v>1</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9" s="14">
-        <v>0</v>
-      </c>
-      <c r="G9" s="14">
-        <v>0</v>
-      </c>
-      <c r="H9" s="14">
-        <v>0</v>
-      </c>
-      <c r="I9" s="14">
-        <v>0</v>
-      </c>
-      <c r="J9" s="14">
-        <v>0</v>
-      </c>
-      <c r="K9" s="14">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1076,7 +897,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -1487,7 +1308,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -2248,7 +2069,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -4409,7 +4230,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>

</xml_diff>

<commit_message>
add indepenent vibration control
</commit_message>
<xml_diff>
--- a/Trials.xlsx
+++ b/Trials.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20397"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26327"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PMDLAB\Documents\Python-Experiments\psychopy-scripts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gesch\Documents\LocalStorage\Lab\Experiment_Codes\psychopy-scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8272A46-601B-4459-8430-39DCADBE017B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6478B99-3E21-4075-9687-A1F784A7312B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="720" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="5" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="27">
   <si>
     <t>trial_num</t>
   </si>
@@ -111,6 +111,13 @@
     <t>Vibration = 1
 No Vibration = 0</t>
   </si>
+  <si>
+    <t>trial_type</t>
+  </si>
+  <si>
+    <t>0=slice
+1=stop</t>
+  </si>
 </sst>
 </file>
 
@@ -185,16 +192,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -530,166 +535,172 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultColWidth="17.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr defaultColWidth="17.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" style="6" customWidth="1"/>
-    <col min="2" max="4" width="17.28515625" style="7"/>
-    <col min="5" max="5" width="17.28515625" style="6"/>
-    <col min="6" max="6" width="20.28515625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="17.28515625" style="7"/>
-    <col min="8" max="9" width="16.140625" style="7" customWidth="1"/>
-    <col min="10" max="12" width="16.140625" style="6" customWidth="1"/>
-    <col min="13" max="16384" width="17.28515625" style="6"/>
+    <col min="1" max="1" width="15.33203125" style="4" customWidth="1"/>
+    <col min="2" max="4" width="17.33203125" style="5"/>
+    <col min="5" max="5" width="17.33203125" style="4"/>
+    <col min="6" max="6" width="20.33203125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" style="5"/>
+    <col min="8" max="9" width="16.109375" style="5" customWidth="1"/>
+    <col min="10" max="12" width="16.109375" style="4" customWidth="1"/>
+    <col min="13" max="16384" width="17.33203125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="9" t="s">
+      <c r="B1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" s="9" t="s">
+      <c r="H1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="L1" s="6" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" s="10" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="M1" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" s="8" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="H2" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J2" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="K2" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="L2" s="13" t="s">
+      <c r="L2" s="11" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
+      <c r="M2" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -701,23 +712,23 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -751,8 +762,11 @@
       <c r="K1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -768,26 +782,29 @@
       <c r="E2">
         <v>0</v>
       </c>
-      <c r="F2" s="14">
-        <v>0</v>
-      </c>
-      <c r="G2" s="14">
-        <v>0</v>
-      </c>
-      <c r="H2" s="14">
-        <v>0</v>
-      </c>
-      <c r="I2" s="14">
-        <v>1</v>
-      </c>
-      <c r="J2" s="14">
+      <c r="F2" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1">
+        <v>1</v>
+      </c>
+      <c r="J2" s="1">
         <v>30</v>
       </c>
-      <c r="K2" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K2" s="1">
+        <v>0</v>
+      </c>
+      <c r="L2" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -803,26 +820,29 @@
       <c r="E3">
         <v>0</v>
       </c>
-      <c r="F3" s="14">
-        <v>0</v>
-      </c>
-      <c r="G3" s="14">
-        <v>0</v>
-      </c>
-      <c r="H3" s="14">
-        <v>0</v>
-      </c>
-      <c r="I3" s="14">
-        <v>1</v>
-      </c>
-      <c r="J3" s="14">
+      <c r="F3" s="1">
+        <v>0</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1">
+        <v>1</v>
+      </c>
+      <c r="J3" s="1">
         <v>30</v>
       </c>
-      <c r="K3" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K3" s="1">
+        <v>0</v>
+      </c>
+      <c r="L3" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -838,26 +858,29 @@
       <c r="E4">
         <v>0</v>
       </c>
-      <c r="F4" s="14">
-        <v>0</v>
-      </c>
-      <c r="G4" s="14">
-        <v>0</v>
-      </c>
-      <c r="H4" s="14">
-        <v>0</v>
-      </c>
-      <c r="I4" s="14">
-        <v>1</v>
-      </c>
-      <c r="J4" s="14">
+      <c r="F4" s="1">
+        <v>0</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1">
+        <v>1</v>
+      </c>
+      <c r="J4" s="1">
         <v>30</v>
       </c>
-      <c r="K4" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K4" s="1">
+        <v>1</v>
+      </c>
+      <c r="L4" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -873,23 +896,26 @@
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="F5" s="14">
-        <v>0</v>
-      </c>
-      <c r="G5" s="14">
-        <v>0</v>
-      </c>
-      <c r="H5" s="14">
-        <v>0</v>
-      </c>
-      <c r="I5" s="14">
-        <v>1</v>
-      </c>
-      <c r="J5" s="14">
+      <c r="F5" s="1">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1">
+        <v>1</v>
+      </c>
+      <c r="J5" s="1">
         <v>30</v>
       </c>
-      <c r="K5" s="14">
-        <v>1</v>
+      <c r="K5" s="1">
+        <v>1</v>
+      </c>
+      <c r="L5" s="12">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -902,23 +928,23 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -952,8 +978,11 @@
       <c r="K1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -966,29 +995,32 @@
       <c r="D2" s="1">
         <v>1</v>
       </c>
-      <c r="E2" s="14">
-        <v>0</v>
-      </c>
-      <c r="F2" s="14">
-        <v>0</v>
-      </c>
-      <c r="G2" s="14">
-        <v>0</v>
-      </c>
-      <c r="H2" s="14">
-        <v>0</v>
-      </c>
-      <c r="I2" s="14">
-        <v>0</v>
-      </c>
-      <c r="J2" s="14">
-        <v>0</v>
-      </c>
-      <c r="K2" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1">
+        <v>0</v>
+      </c>
+      <c r="L2" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1001,29 +1033,32 @@
       <c r="D3" s="1">
         <v>1</v>
       </c>
-      <c r="E3" s="14">
-        <v>0</v>
-      </c>
-      <c r="F3" s="14">
-        <v>0</v>
-      </c>
-      <c r="G3" s="14">
-        <v>0</v>
-      </c>
-      <c r="H3" s="14">
-        <v>0</v>
-      </c>
-      <c r="I3" s="14">
-        <v>0</v>
-      </c>
-      <c r="J3" s="14">
-        <v>0</v>
-      </c>
-      <c r="K3" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E3" s="1">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0</v>
+      </c>
+      <c r="J3" s="1">
+        <v>0</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0</v>
+      </c>
+      <c r="L3" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1036,29 +1071,32 @@
       <c r="D4" s="1">
         <v>1</v>
       </c>
-      <c r="E4" s="14">
-        <v>0</v>
-      </c>
-      <c r="F4" s="14">
-        <v>0</v>
-      </c>
-      <c r="G4" s="14">
-        <v>0</v>
-      </c>
-      <c r="H4" s="14">
-        <v>0</v>
-      </c>
-      <c r="I4" s="14">
-        <v>0</v>
-      </c>
-      <c r="J4" s="14">
-        <v>0</v>
-      </c>
-      <c r="K4" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E4" s="1">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1">
+        <v>0</v>
+      </c>
+      <c r="J4" s="1">
+        <v>0</v>
+      </c>
+      <c r="K4" s="1">
+        <v>0</v>
+      </c>
+      <c r="L4" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1071,29 +1109,32 @@
       <c r="D5" s="1">
         <v>1</v>
       </c>
-      <c r="E5" s="14">
-        <v>0</v>
-      </c>
-      <c r="F5" s="14">
-        <v>0</v>
-      </c>
-      <c r="G5" s="14">
-        <v>0</v>
-      </c>
-      <c r="H5" s="14">
-        <v>0</v>
-      </c>
-      <c r="I5" s="14">
-        <v>0</v>
-      </c>
-      <c r="J5" s="14">
-        <v>0</v>
-      </c>
-      <c r="K5" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E5" s="1">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0</v>
+      </c>
+      <c r="J5" s="1">
+        <v>0</v>
+      </c>
+      <c r="K5" s="1">
+        <v>0</v>
+      </c>
+      <c r="L5" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1106,29 +1147,29 @@
       <c r="D6" s="1">
         <v>1</v>
       </c>
-      <c r="E6" s="14">
-        <v>0</v>
-      </c>
-      <c r="F6" s="14">
-        <v>0</v>
-      </c>
-      <c r="G6" s="14">
-        <v>0</v>
-      </c>
-      <c r="H6" s="14">
-        <v>0</v>
-      </c>
-      <c r="I6" s="14">
-        <v>0</v>
-      </c>
-      <c r="J6" s="14">
-        <v>0</v>
-      </c>
-      <c r="K6" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E6" s="1">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1">
+        <v>0</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0</v>
+      </c>
+      <c r="I6" s="1">
+        <v>0</v>
+      </c>
+      <c r="J6" s="1">
+        <v>0</v>
+      </c>
+      <c r="K6" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1141,29 +1182,29 @@
       <c r="D7" s="1">
         <v>1</v>
       </c>
-      <c r="E7" s="14">
-        <v>0</v>
-      </c>
-      <c r="F7" s="14">
-        <v>0</v>
-      </c>
-      <c r="G7" s="14">
-        <v>0</v>
-      </c>
-      <c r="H7" s="14">
-        <v>0</v>
-      </c>
-      <c r="I7" s="14">
-        <v>0</v>
-      </c>
-      <c r="J7" s="14">
-        <v>0</v>
-      </c>
-      <c r="K7" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E7" s="1">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0</v>
+      </c>
+      <c r="I7" s="1">
+        <v>0</v>
+      </c>
+      <c r="J7" s="1">
+        <v>0</v>
+      </c>
+      <c r="K7" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1176,29 +1217,29 @@
       <c r="D8" s="1">
         <v>1</v>
       </c>
-      <c r="E8" s="14">
-        <v>0</v>
-      </c>
-      <c r="F8" s="14">
-        <v>0</v>
-      </c>
-      <c r="G8" s="14">
-        <v>0</v>
-      </c>
-      <c r="H8" s="14">
-        <v>0</v>
-      </c>
-      <c r="I8" s="14">
-        <v>0</v>
-      </c>
-      <c r="J8" s="14">
-        <v>0</v>
-      </c>
-      <c r="K8" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E8" s="1">
+        <v>0</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0</v>
+      </c>
+      <c r="G8" s="1">
+        <v>0</v>
+      </c>
+      <c r="H8" s="1">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1">
+        <v>0</v>
+      </c>
+      <c r="J8" s="1">
+        <v>0</v>
+      </c>
+      <c r="K8" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1211,29 +1252,29 @@
       <c r="D9" s="1">
         <v>1</v>
       </c>
-      <c r="E9" s="14">
-        <v>0</v>
-      </c>
-      <c r="F9" s="14">
-        <v>0</v>
-      </c>
-      <c r="G9" s="14">
-        <v>0</v>
-      </c>
-      <c r="H9" s="14">
-        <v>0</v>
-      </c>
-      <c r="I9" s="14">
-        <v>0</v>
-      </c>
-      <c r="J9" s="14">
-        <v>0</v>
-      </c>
-      <c r="K9" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E9" s="1">
+        <v>0</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0</v>
+      </c>
+      <c r="G9" s="1">
+        <v>0</v>
+      </c>
+      <c r="H9" s="1">
+        <v>0</v>
+      </c>
+      <c r="I9" s="1">
+        <v>0</v>
+      </c>
+      <c r="J9" s="1">
+        <v>0</v>
+      </c>
+      <c r="K9" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1246,29 +1287,29 @@
       <c r="D10" s="1">
         <v>1</v>
       </c>
-      <c r="E10" s="14">
-        <v>0</v>
-      </c>
-      <c r="F10" s="14">
-        <v>0</v>
-      </c>
-      <c r="G10" s="14">
-        <v>0</v>
-      </c>
-      <c r="H10" s="14">
-        <v>0</v>
-      </c>
-      <c r="I10" s="14">
-        <v>0</v>
-      </c>
-      <c r="J10" s="14">
-        <v>0</v>
-      </c>
-      <c r="K10" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E10" s="1">
+        <v>0</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0</v>
+      </c>
+      <c r="G10" s="1">
+        <v>0</v>
+      </c>
+      <c r="H10" s="1">
+        <v>0</v>
+      </c>
+      <c r="I10" s="1">
+        <v>0</v>
+      </c>
+      <c r="J10" s="1">
+        <v>0</v>
+      </c>
+      <c r="K10" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1281,25 +1322,25 @@
       <c r="D11" s="1">
         <v>1</v>
       </c>
-      <c r="E11" s="14">
-        <v>0</v>
-      </c>
-      <c r="F11" s="14">
-        <v>0</v>
-      </c>
-      <c r="G11" s="14">
-        <v>0</v>
-      </c>
-      <c r="H11" s="14">
-        <v>0</v>
-      </c>
-      <c r="I11" s="14">
-        <v>0</v>
-      </c>
-      <c r="J11" s="14">
-        <v>0</v>
-      </c>
-      <c r="K11" s="14">
+      <c r="E11" s="1">
+        <v>0</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0</v>
+      </c>
+      <c r="G11" s="1">
+        <v>0</v>
+      </c>
+      <c r="H11" s="1">
+        <v>0</v>
+      </c>
+      <c r="I11" s="1">
+        <v>0</v>
+      </c>
+      <c r="J11" s="1">
+        <v>0</v>
+      </c>
+      <c r="K11" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1313,23 +1354,23 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1363,8 +1404,11 @@
       <c r="K1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1377,29 +1421,32 @@
       <c r="D2" s="1">
         <v>0</v>
       </c>
-      <c r="E2" s="14">
-        <v>0</v>
-      </c>
-      <c r="F2" s="14">
-        <v>0</v>
-      </c>
-      <c r="G2" s="14">
-        <v>0</v>
-      </c>
-      <c r="H2" s="14">
-        <v>0</v>
-      </c>
-      <c r="I2" s="14">
-        <v>0</v>
-      </c>
-      <c r="J2" s="14">
-        <v>0</v>
-      </c>
-      <c r="K2" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1">
+        <v>0</v>
+      </c>
+      <c r="L2" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1412,29 +1459,32 @@
       <c r="D3" s="1">
         <v>0</v>
       </c>
-      <c r="E3" s="14">
-        <v>0</v>
-      </c>
-      <c r="F3" s="14">
-        <v>0</v>
-      </c>
-      <c r="G3" s="14">
-        <v>0</v>
-      </c>
-      <c r="H3" s="14">
-        <v>0</v>
-      </c>
-      <c r="I3" s="14">
-        <v>0</v>
-      </c>
-      <c r="J3" s="14">
-        <v>0</v>
-      </c>
-      <c r="K3" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E3" s="1">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0</v>
+      </c>
+      <c r="J3" s="1">
+        <v>0</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0</v>
+      </c>
+      <c r="L3" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1447,29 +1497,32 @@
       <c r="D4" s="1">
         <v>0</v>
       </c>
-      <c r="E4" s="14">
-        <v>0</v>
-      </c>
-      <c r="F4" s="14">
-        <v>0</v>
-      </c>
-      <c r="G4" s="14">
-        <v>0</v>
-      </c>
-      <c r="H4" s="14">
-        <v>0</v>
-      </c>
-      <c r="I4" s="14">
-        <v>0</v>
-      </c>
-      <c r="J4" s="14">
-        <v>0</v>
-      </c>
-      <c r="K4" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E4" s="1">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1">
+        <v>0</v>
+      </c>
+      <c r="J4" s="1">
+        <v>0</v>
+      </c>
+      <c r="K4" s="1">
+        <v>0</v>
+      </c>
+      <c r="L4" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1482,29 +1535,32 @@
       <c r="D5" s="1">
         <v>0</v>
       </c>
-      <c r="E5" s="14">
-        <v>0</v>
-      </c>
-      <c r="F5" s="14">
-        <v>0</v>
-      </c>
-      <c r="G5" s="14">
-        <v>0</v>
-      </c>
-      <c r="H5" s="14">
-        <v>0</v>
-      </c>
-      <c r="I5" s="14">
-        <v>0</v>
-      </c>
-      <c r="J5" s="14">
-        <v>0</v>
-      </c>
-      <c r="K5" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E5" s="1">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0</v>
+      </c>
+      <c r="J5" s="1">
+        <v>0</v>
+      </c>
+      <c r="K5" s="1">
+        <v>0</v>
+      </c>
+      <c r="L5" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1517,29 +1573,29 @@
       <c r="D6" s="1">
         <v>0</v>
       </c>
-      <c r="E6" s="14">
-        <v>0</v>
-      </c>
-      <c r="F6" s="14">
-        <v>0</v>
-      </c>
-      <c r="G6" s="14">
-        <v>0</v>
-      </c>
-      <c r="H6" s="14">
-        <v>0</v>
-      </c>
-      <c r="I6" s="14">
-        <v>0</v>
-      </c>
-      <c r="J6" s="14">
-        <v>0</v>
-      </c>
-      <c r="K6" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E6" s="1">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1">
+        <v>0</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0</v>
+      </c>
+      <c r="I6" s="1">
+        <v>0</v>
+      </c>
+      <c r="J6" s="1">
+        <v>0</v>
+      </c>
+      <c r="K6" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1552,29 +1608,29 @@
       <c r="D7" s="1">
         <v>0</v>
       </c>
-      <c r="E7" s="14">
-        <v>0</v>
-      </c>
-      <c r="F7" s="14">
-        <v>0</v>
-      </c>
-      <c r="G7" s="14">
-        <v>0</v>
-      </c>
-      <c r="H7" s="14">
-        <v>0</v>
-      </c>
-      <c r="I7" s="14">
-        <v>0</v>
-      </c>
-      <c r="J7" s="14">
-        <v>0</v>
-      </c>
-      <c r="K7" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E7" s="1">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0</v>
+      </c>
+      <c r="I7" s="1">
+        <v>0</v>
+      </c>
+      <c r="J7" s="1">
+        <v>0</v>
+      </c>
+      <c r="K7" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1587,29 +1643,29 @@
       <c r="D8" s="1">
         <v>0</v>
       </c>
-      <c r="E8" s="14">
-        <v>0</v>
-      </c>
-      <c r="F8" s="14">
-        <v>0</v>
-      </c>
-      <c r="G8" s="14">
-        <v>0</v>
-      </c>
-      <c r="H8" s="14">
-        <v>0</v>
-      </c>
-      <c r="I8" s="14">
-        <v>0</v>
-      </c>
-      <c r="J8" s="14">
-        <v>0</v>
-      </c>
-      <c r="K8" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E8" s="1">
+        <v>0</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0</v>
+      </c>
+      <c r="G8" s="1">
+        <v>0</v>
+      </c>
+      <c r="H8" s="1">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1">
+        <v>0</v>
+      </c>
+      <c r="J8" s="1">
+        <v>0</v>
+      </c>
+      <c r="K8" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1622,29 +1678,29 @@
       <c r="D9" s="1">
         <v>0</v>
       </c>
-      <c r="E9" s="14">
-        <v>0</v>
-      </c>
-      <c r="F9" s="14">
-        <v>0</v>
-      </c>
-      <c r="G9" s="14">
-        <v>0</v>
-      </c>
-      <c r="H9" s="14">
-        <v>0</v>
-      </c>
-      <c r="I9" s="14">
-        <v>0</v>
-      </c>
-      <c r="J9" s="14">
-        <v>0</v>
-      </c>
-      <c r="K9" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E9" s="1">
+        <v>0</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0</v>
+      </c>
+      <c r="G9" s="1">
+        <v>0</v>
+      </c>
+      <c r="H9" s="1">
+        <v>0</v>
+      </c>
+      <c r="I9" s="1">
+        <v>0</v>
+      </c>
+      <c r="J9" s="1">
+        <v>0</v>
+      </c>
+      <c r="K9" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1657,29 +1713,29 @@
       <c r="D10" s="1">
         <v>0</v>
       </c>
-      <c r="E10" s="14">
-        <v>0</v>
-      </c>
-      <c r="F10" s="14">
-        <v>0</v>
-      </c>
-      <c r="G10" s="14">
-        <v>0</v>
-      </c>
-      <c r="H10" s="14">
-        <v>0</v>
-      </c>
-      <c r="I10" s="14">
-        <v>0</v>
-      </c>
-      <c r="J10" s="14">
-        <v>0</v>
-      </c>
-      <c r="K10" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E10" s="1">
+        <v>0</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0</v>
+      </c>
+      <c r="G10" s="1">
+        <v>0</v>
+      </c>
+      <c r="H10" s="1">
+        <v>0</v>
+      </c>
+      <c r="I10" s="1">
+        <v>0</v>
+      </c>
+      <c r="J10" s="1">
+        <v>0</v>
+      </c>
+      <c r="K10" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1692,29 +1748,29 @@
       <c r="D11" s="1">
         <v>0</v>
       </c>
-      <c r="E11" s="14">
-        <v>0</v>
-      </c>
-      <c r="F11" s="14">
-        <v>0</v>
-      </c>
-      <c r="G11" s="14">
-        <v>0</v>
-      </c>
-      <c r="H11" s="14">
-        <v>0</v>
-      </c>
-      <c r="I11" s="14">
-        <v>0</v>
-      </c>
-      <c r="J11" s="14">
-        <v>0</v>
-      </c>
-      <c r="K11" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E11" s="1">
+        <v>0</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0</v>
+      </c>
+      <c r="G11" s="1">
+        <v>0</v>
+      </c>
+      <c r="H11" s="1">
+        <v>0</v>
+      </c>
+      <c r="I11" s="1">
+        <v>0</v>
+      </c>
+      <c r="J11" s="1">
+        <v>0</v>
+      </c>
+      <c r="K11" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>1</v>
       </c>
@@ -1727,29 +1783,29 @@
       <c r="D12" s="1">
         <v>0</v>
       </c>
-      <c r="E12" s="14">
-        <v>0</v>
-      </c>
-      <c r="F12" s="14">
-        <v>0</v>
-      </c>
-      <c r="G12" s="14">
-        <v>0</v>
-      </c>
-      <c r="H12" s="14">
-        <v>0</v>
-      </c>
-      <c r="I12" s="14">
-        <v>0</v>
-      </c>
-      <c r="J12" s="14">
-        <v>0</v>
-      </c>
-      <c r="K12" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E12" s="1">
+        <v>0</v>
+      </c>
+      <c r="F12" s="1">
+        <v>0</v>
+      </c>
+      <c r="G12" s="1">
+        <v>0</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0</v>
+      </c>
+      <c r="I12" s="1">
+        <v>0</v>
+      </c>
+      <c r="J12" s="1">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>2</v>
       </c>
@@ -1762,29 +1818,29 @@
       <c r="D13" s="1">
         <v>0</v>
       </c>
-      <c r="E13" s="14">
-        <v>0</v>
-      </c>
-      <c r="F13" s="14">
-        <v>0</v>
-      </c>
-      <c r="G13" s="14">
-        <v>0</v>
-      </c>
-      <c r="H13" s="14">
-        <v>0</v>
-      </c>
-      <c r="I13" s="14">
-        <v>0</v>
-      </c>
-      <c r="J13" s="14">
-        <v>0</v>
-      </c>
-      <c r="K13" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0</v>
+      </c>
+      <c r="G13" s="1">
+        <v>0</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1">
+        <v>0</v>
+      </c>
+      <c r="J13" s="1">
+        <v>0</v>
+      </c>
+      <c r="K13" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>3</v>
       </c>
@@ -1797,29 +1853,29 @@
       <c r="D14" s="1">
         <v>0</v>
       </c>
-      <c r="E14" s="14">
-        <v>0</v>
-      </c>
-      <c r="F14" s="14">
-        <v>0</v>
-      </c>
-      <c r="G14" s="14">
-        <v>0</v>
-      </c>
-      <c r="H14" s="14">
-        <v>0</v>
-      </c>
-      <c r="I14" s="14">
-        <v>0</v>
-      </c>
-      <c r="J14" s="14">
-        <v>0</v>
-      </c>
-      <c r="K14" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E14" s="1">
+        <v>0</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0</v>
+      </c>
+      <c r="G14" s="1">
+        <v>0</v>
+      </c>
+      <c r="H14" s="1">
+        <v>0</v>
+      </c>
+      <c r="I14" s="1">
+        <v>0</v>
+      </c>
+      <c r="J14" s="1">
+        <v>0</v>
+      </c>
+      <c r="K14" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>4</v>
       </c>
@@ -1832,29 +1888,29 @@
       <c r="D15" s="1">
         <v>0</v>
       </c>
-      <c r="E15" s="14">
-        <v>0</v>
-      </c>
-      <c r="F15" s="14">
-        <v>0</v>
-      </c>
-      <c r="G15" s="14">
-        <v>0</v>
-      </c>
-      <c r="H15" s="14">
-        <v>0</v>
-      </c>
-      <c r="I15" s="14">
-        <v>0</v>
-      </c>
-      <c r="J15" s="14">
-        <v>0</v>
-      </c>
-      <c r="K15" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E15" s="1">
+        <v>0</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0</v>
+      </c>
+      <c r="G15" s="1">
+        <v>0</v>
+      </c>
+      <c r="H15" s="1">
+        <v>0</v>
+      </c>
+      <c r="I15" s="1">
+        <v>0</v>
+      </c>
+      <c r="J15" s="1">
+        <v>0</v>
+      </c>
+      <c r="K15" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>5</v>
       </c>
@@ -1867,29 +1923,29 @@
       <c r="D16" s="1">
         <v>0</v>
       </c>
-      <c r="E16" s="14">
-        <v>0</v>
-      </c>
-      <c r="F16" s="14">
-        <v>0</v>
-      </c>
-      <c r="G16" s="14">
-        <v>0</v>
-      </c>
-      <c r="H16" s="14">
-        <v>0</v>
-      </c>
-      <c r="I16" s="14">
-        <v>0</v>
-      </c>
-      <c r="J16" s="14">
-        <v>0</v>
-      </c>
-      <c r="K16" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E16" s="1">
+        <v>0</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0</v>
+      </c>
+      <c r="G16" s="1">
+        <v>0</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0</v>
+      </c>
+      <c r="I16" s="1">
+        <v>0</v>
+      </c>
+      <c r="J16" s="1">
+        <v>0</v>
+      </c>
+      <c r="K16" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>6</v>
       </c>
@@ -1902,29 +1958,29 @@
       <c r="D17" s="1">
         <v>0</v>
       </c>
-      <c r="E17" s="14">
-        <v>0</v>
-      </c>
-      <c r="F17" s="14">
-        <v>0</v>
-      </c>
-      <c r="G17" s="14">
-        <v>0</v>
-      </c>
-      <c r="H17" s="14">
-        <v>0</v>
-      </c>
-      <c r="I17" s="14">
-        <v>0</v>
-      </c>
-      <c r="J17" s="14">
-        <v>0</v>
-      </c>
-      <c r="K17" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E17" s="1">
+        <v>0</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0</v>
+      </c>
+      <c r="G17" s="1">
+        <v>0</v>
+      </c>
+      <c r="H17" s="1">
+        <v>0</v>
+      </c>
+      <c r="I17" s="1">
+        <v>0</v>
+      </c>
+      <c r="J17" s="1">
+        <v>0</v>
+      </c>
+      <c r="K17" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>7</v>
       </c>
@@ -1937,29 +1993,29 @@
       <c r="D18" s="1">
         <v>0</v>
       </c>
-      <c r="E18" s="14">
-        <v>0</v>
-      </c>
-      <c r="F18" s="14">
-        <v>0</v>
-      </c>
-      <c r="G18" s="14">
-        <v>0</v>
-      </c>
-      <c r="H18" s="14">
-        <v>0</v>
-      </c>
-      <c r="I18" s="14">
-        <v>0</v>
-      </c>
-      <c r="J18" s="14">
-        <v>0</v>
-      </c>
-      <c r="K18" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E18" s="1">
+        <v>0</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0</v>
+      </c>
+      <c r="G18" s="1">
+        <v>0</v>
+      </c>
+      <c r="H18" s="1">
+        <v>0</v>
+      </c>
+      <c r="I18" s="1">
+        <v>0</v>
+      </c>
+      <c r="J18" s="1">
+        <v>0</v>
+      </c>
+      <c r="K18" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>8</v>
       </c>
@@ -1972,29 +2028,29 @@
       <c r="D19" s="1">
         <v>0</v>
       </c>
-      <c r="E19" s="14">
-        <v>0</v>
-      </c>
-      <c r="F19" s="14">
-        <v>0</v>
-      </c>
-      <c r="G19" s="14">
-        <v>0</v>
-      </c>
-      <c r="H19" s="14">
-        <v>0</v>
-      </c>
-      <c r="I19" s="14">
-        <v>0</v>
-      </c>
-      <c r="J19" s="14">
-        <v>0</v>
-      </c>
-      <c r="K19" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E19" s="1">
+        <v>0</v>
+      </c>
+      <c r="F19" s="1">
+        <v>0</v>
+      </c>
+      <c r="G19" s="1">
+        <v>0</v>
+      </c>
+      <c r="H19" s="1">
+        <v>0</v>
+      </c>
+      <c r="I19" s="1">
+        <v>0</v>
+      </c>
+      <c r="J19" s="1">
+        <v>0</v>
+      </c>
+      <c r="K19" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>9</v>
       </c>
@@ -2007,29 +2063,29 @@
       <c r="D20" s="1">
         <v>0</v>
       </c>
-      <c r="E20" s="14">
-        <v>0</v>
-      </c>
-      <c r="F20" s="14">
-        <v>0</v>
-      </c>
-      <c r="G20" s="14">
-        <v>0</v>
-      </c>
-      <c r="H20" s="14">
-        <v>0</v>
-      </c>
-      <c r="I20" s="14">
-        <v>0</v>
-      </c>
-      <c r="J20" s="14">
-        <v>0</v>
-      </c>
-      <c r="K20" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E20" s="1">
+        <v>0</v>
+      </c>
+      <c r="F20" s="1">
+        <v>0</v>
+      </c>
+      <c r="G20" s="1">
+        <v>0</v>
+      </c>
+      <c r="H20" s="1">
+        <v>0</v>
+      </c>
+      <c r="I20" s="1">
+        <v>0</v>
+      </c>
+      <c r="J20" s="1">
+        <v>0</v>
+      </c>
+      <c r="K20" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>10</v>
       </c>
@@ -2042,25 +2098,25 @@
       <c r="D21" s="1">
         <v>0</v>
       </c>
-      <c r="E21" s="14">
-        <v>0</v>
-      </c>
-      <c r="F21" s="14">
-        <v>0</v>
-      </c>
-      <c r="G21" s="14">
-        <v>0</v>
-      </c>
-      <c r="H21" s="14">
-        <v>0</v>
-      </c>
-      <c r="I21" s="14">
-        <v>0</v>
-      </c>
-      <c r="J21" s="14">
-        <v>0</v>
-      </c>
-      <c r="K21" s="14">
+      <c r="E21" s="1">
+        <v>0</v>
+      </c>
+      <c r="F21" s="1">
+        <v>0</v>
+      </c>
+      <c r="G21" s="1">
+        <v>0</v>
+      </c>
+      <c r="H21" s="1">
+        <v>0</v>
+      </c>
+      <c r="I21" s="1">
+        <v>0</v>
+      </c>
+      <c r="J21" s="1">
+        <v>0</v>
+      </c>
+      <c r="K21" s="1">
         <v>0</v>
       </c>
     </row>
@@ -2074,23 +2130,23 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L61"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2124,8 +2180,11 @@
       <c r="K1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -2159,8 +2218,11 @@
       <c r="K2" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L2" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -2194,8 +2256,11 @@
       <c r="K3" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -2229,8 +2294,11 @@
       <c r="K4" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L4" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -2264,8 +2332,11 @@
       <c r="K5" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -2300,7 +2371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -2335,7 +2406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -2370,7 +2441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -2405,7 +2476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -2440,7 +2511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -2475,7 +2546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -2510,7 +2581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2545,7 +2616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -2580,7 +2651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -2615,7 +2686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -2650,7 +2721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -2685,7 +2756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -2720,7 +2791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -2755,7 +2826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -2790,7 +2861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -2825,7 +2896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -2860,7 +2931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -2895,7 +2966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -2930,7 +3001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -2965,7 +3036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -3000,7 +3071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -3035,7 +3106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -3070,7 +3141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -3105,7 +3176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -3140,7 +3211,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -3175,7 +3246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -3210,7 +3281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -3245,7 +3316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -3280,7 +3351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -3315,7 +3386,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -3350,7 +3421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -3385,7 +3456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -3420,7 +3491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -3455,7 +3526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -3490,7 +3561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -3525,7 +3596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -3560,7 +3631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -3595,7 +3666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -3630,7 +3701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -3665,7 +3736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -3700,7 +3771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -3735,7 +3806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -3770,7 +3841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -3805,7 +3876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -3840,7 +3911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -3875,7 +3946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52" s="1">
         <v>51</v>
       </c>
@@ -3910,7 +3981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -3945,7 +4016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -3980,7 +4051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -4015,7 +4086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -4050,7 +4121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57" s="1">
         <v>56</v>
       </c>
@@ -4085,7 +4156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58" s="1">
         <v>57</v>
       </c>
@@ -4120,7 +4191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" s="1">
         <v>58</v>
       </c>
@@ -4155,7 +4226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -4190,7 +4261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -4235,23 +4306,23 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4285,12 +4356,15 @@
       <c r="K1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="1">
@@ -4302,12 +4376,15 @@
       <c r="E2" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L2" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="1">
@@ -4319,12 +4396,15 @@
       <c r="E3" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="1">
@@ -4336,12 +4416,15 @@
       <c r="E4" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L4" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="1">
@@ -4353,12 +4436,15 @@
       <c r="E5" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="1">
@@ -4371,11 +4457,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="1">
@@ -4388,11 +4474,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>4</v>
       </c>
       <c r="C8" s="1">
@@ -4405,11 +4491,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="1">
@@ -4422,11 +4508,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>4</v>
       </c>
       <c r="C10" s="1">
@@ -4439,11 +4525,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" t="s">
         <v>4</v>
       </c>
       <c r="C11" s="1">
@@ -4456,11 +4542,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
         <v>4</v>
       </c>
       <c r="C12" s="1">
@@ -4473,11 +4559,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" t="s">
         <v>4</v>
       </c>
       <c r="C13" s="1">
@@ -4490,11 +4576,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" t="s">
         <v>4</v>
       </c>
       <c r="C14" s="1">
@@ -4507,11 +4593,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" t="s">
         <v>4</v>
       </c>
       <c r="C15" s="1">
@@ -4524,11 +4610,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" t="s">
         <v>4</v>
       </c>
       <c r="C16" s="1">
@@ -4541,11 +4627,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" t="s">
         <v>4</v>
       </c>
       <c r="C17" s="1">
@@ -4558,11 +4644,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" t="s">
         <v>4</v>
       </c>
       <c r="C18" s="1">
@@ -4575,11 +4661,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" t="s">
         <v>4</v>
       </c>
       <c r="C19" s="1">
@@ -4592,11 +4678,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" t="s">
         <v>4</v>
       </c>
       <c r="C20" s="1">
@@ -4609,11 +4695,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" t="s">
         <v>4</v>
       </c>
       <c r="C21" s="1">

</xml_diff>